<commit_message>
Bilanz: Name → Rolle zählt nicht als Änderung; alle offenen Bitten je Prüfer gebündelt (E-197 Nachtrag)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WbXnSzce2P68GngQY2h6hr
</commit_message>
<xml_diff>
--- a/docs/freigabe-katalog/versand-2026-10-25-nachpruefung/steuern/Betriebsklar-Nachpruefliste-Steuerberater.xlsx
+++ b/docs/freigabe-katalog/versand-2026-10-25-nachpruefung/steuern/Betriebsklar-Nachpruefliste-Steuerberater.xlsx
@@ -527,7 +527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -684,67 +684,35 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Vorlage</t>
+          <t>Nennung im Vermerk</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>bilanz_guv</t>
+          <t>alle</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>a266993aadfd</t>
+          <t>–</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Bilanz und Gewinn- und Verlustrechnung</t>
+          <t>Rolle statt Name</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Seit Ihrer Freigabe geändert sind nur diese Varianten: Hilfetext eines Formularfelds: „Steuerberater“ statt Ihres Namens (das gedruckte Dokument ist unverändert). Die übrigen 29 von 30 Varianten (Rechtsformen, Länder, Kleinunternehmer) sind unverändert; für sie gilt Ihre Freigabe weiter, die App zeigt dort den Vermerk. Bitte sehen Sie die geänderten Varianten durch und bestätigen Sie sie per E-Mail.</t>
+          <t>Die App nennt Personen nicht mehr. Bisher mit Ihrem Namen und der Kanzlei (Ihre Bestätigung vom 23.10.2026); künftig nennt der Vermerk Ihre Rolle: „Fachlich durchgesehen von einem Steuerberater (Stand …) – ohne Gewähr für den Einzelfall.“ (bei Einschränkungen mit dem Zusatz in Klammern, bei offenen Punkten „teilweise“). Bitte bestätigen Sie per E-Mail, dass die Nennung der Rolle so in Ordnung ist.</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr"/>
       <c r="H5" s="3" t="inlineStr"/>
     </row>
-    <row r="6">
-      <c r="A6" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Nennung im Vermerk</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>alle</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>Rolle statt Name</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>Die App nennt Personen nicht mehr. Bisher mit Ihrem Namen und der Kanzlei (Ihre Bestätigung vom 23.10.2026); künftig nennt der Vermerk Ihre Rolle: „Fachlich durchgesehen von einem Steuerberater (Stand …) – ohne Gewähr für den Einzelfall.“ (bei Einschränkungen mit dem Zusatz in Klammern, bei offenen Punkten „teilweise“). Bitte bestätigen Sie per E-Mail, dass die Nennung der Rolle so in Ordnung ist.</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr"/>
-      <c r="H6" s="3" t="inlineStr"/>
-    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="G2:G6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G2:G5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"bestätigt,ändern (Anmerkung),nicht mein Bereich"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>